<commit_message>
Correcion menor en Reclamos
</commit_message>
<xml_diff>
--- a/Modificaciones solicitadas.xlsx
+++ b/Modificaciones solicitadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Xamarin\RowingApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B00E9A-86B4-4BF1-A301-BA6815EF3731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231CB6F1-8FAE-45BD-9717-0BC2FC884140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2D167E44-E563-4DF9-9CAD-3636B941BCB8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>Fecha</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t>Poner menu Reclamos y sacarlo de Obras. Que se pueda elegir la Obra (serán 2, en Tabla Obras las que tienen HabilitaReclamosAPP = 1 y módulo = al del usuario logueado)</t>
+  </si>
+  <si>
+    <t>20/12/2021 V.6</t>
   </si>
 </sst>
 </file>
@@ -821,9 +824,13 @@
       <c r="B18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="6"/>
+      <c r="C18" s="10">
+        <v>44546</v>
+      </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="3"/>
+      <c r="E18" s="9" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>

</xml_diff>

<commit_message>
Agregado de una opcion de Tipo de Foto en Obras
</commit_message>
<xml_diff>
--- a/Modificaciones solicitadas.xlsx
+++ b/Modificaciones solicitadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Xamarin\RowingApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBEAA16-7F52-4BCF-A153-79D595FD089E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75748FAA-5471-4388-AC7B-03B719E2AB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2D167E44-E563-4DF9-9CAD-3636B941BCB8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>Fecha</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>Poder subir fotos de la galería</t>
+  </si>
+  <si>
+    <t>Agregar en Obras como opción de foto "Vereda conforme". Ponerlo antes de "Finalización del trabajo"</t>
   </si>
 </sst>
 </file>
@@ -845,7 +848,9 @@
       <c r="B19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="6"/>
+      <c r="C19" s="10">
+        <v>44550</v>
+      </c>
       <c r="D19" s="5"/>
       <c r="E19" s="3"/>
     </row>
@@ -856,14 +861,22 @@
       <c r="B20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="6"/>
+      <c r="C20" s="10">
+        <v>44550</v>
+      </c>
       <c r="D20" s="5"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="6"/>
+    <row r="21" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <v>44552</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="10">
+        <v>44552</v>
+      </c>
       <c r="D21" s="5"/>
       <c r="E21" s="3"/>
     </row>

</xml_diff>

<commit_message>
GetObra en API Account
</commit_message>
<xml_diff>
--- a/Modificaciones solicitadas.xlsx
+++ b/Modificaciones solicitadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Xamarin\RowingApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75748FAA-5471-4388-AC7B-03B719E2AB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D29D31-7A7E-404E-ADDA-E64DAED2F15D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2D167E44-E563-4DF9-9CAD-3636B941BCB8}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
   <si>
     <t>Fecha</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>Agregar en Obras como opción de foto "Vereda conforme". Ponerlo antes de "Finalización del trabajo"</t>
+  </si>
+  <si>
+    <t>27/12/2021 V.7</t>
   </si>
 </sst>
 </file>
@@ -852,7 +855,9 @@
         <v>44550</v>
       </c>
       <c r="D19" s="5"/>
-      <c r="E19" s="3"/>
+      <c r="E19" s="9" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
@@ -865,7 +870,9 @@
         <v>44550</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="3"/>
+      <c r="E20" s="9" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="21" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
@@ -878,7 +885,9 @@
         <v>44552</v>
       </c>
       <c r="D21" s="5"/>
-      <c r="E21" s="3"/>
+      <c r="E21" s="9" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>

</xml_diff>